<commit_message>
Site gaps: WKND non-breaking spaces, magazine footer spacing, compact article sidebars
- importer: WKND's non-breaking spaces decide where lines wrap ("the&nbsp;
  quintessential"); the importer's DOM had lost them and the markdown step
  drops them. wknd-cleanup restores them from the raw HTML and carries them
  as U+202F; upload-to-da.mjs writes them back as &nbsp; (Edge Delivery
  keeps &nbsp; from DA). Fixes the reflow gaps on LA skateparks and Tahoe.
- magazine: Template metadata, 48px before the footer, members-only cards
  14px under the image, as on the source
- articles without WKND's hidden sidebar spacer (arctic surfing, ski
  touring) get the extra section style "compact" (36px less under
  "Share this story")

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-about.report.xlsx
+++ b/tools/importer/reports/import-about.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="122">
   <si>
     <t>_reportFile</t>
   </si>
@@ -58,7 +58,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-09-28T05:59:23.894Z</t>
+    <t>2026-09-28T08:40:28.985Z</t>
   </si>
   <si>
     <t>WKND Adventures and Travel</t>
@@ -82,7 +82,7 @@
     <t>about</t>
   </si>
   <si>
-    <t>2026-09-28T06:49:29.123Z</t>
+    <t>2026-09-28T08:42:15.364Z</t>
   </si>
   <si>
     <t>About Us</t>
@@ -103,7 +103,7 @@
     <t>adventure-listing</t>
   </si>
   <si>
-    <t>2026-09-28T06:21:34.372Z</t>
+    <t>2026-09-28T08:42:00.642Z</t>
   </si>
   <si>
     <t>Adventures</t>
@@ -124,7 +124,7 @@
     <t>faq</t>
   </si>
   <si>
-    <t>2026-09-28T06:37:54.159Z</t>
+    <t>2026-09-28T08:42:07.878Z</t>
   </si>
   <si>
     <t>FAQs</t>
@@ -145,7 +145,7 @@
     <t>magazine</t>
   </si>
   <si>
-    <t>2026-09-28T05:59:30.781Z</t>
+    <t>2026-09-28T08:40:37.145Z</t>
   </si>
   <si>
     <t>Magazine</t>
@@ -154,22 +154,37 @@
     <t>https://wknd.site/us/en/magazine.html</t>
   </si>
   <si>
+    <t>us/en/adventures/bali-surf-camp.report.json</t>
+  </si>
+  <si>
+    <t>["carousel-hero","cards-related","tabs"]</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp</t>
+  </si>
+  <si>
+    <t>adventure</t>
+  </si>
+  <si>
+    <t>2026-09-28T08:41:52.456Z</t>
+  </si>
+  <si>
+    <t>Bali Surf Camp</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
+  </si>
+  <si>
     <t>us/en/adventures/climbing-new-zealand.report.json</t>
   </si>
   <si>
     <t>["What to Bring — empty alt, used tab label"]</t>
   </si>
   <si>
-    <t>["carousel-hero","cards-related","tabs"]</t>
-  </si>
-  <si>
     <t>us/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>adventure</t>
-  </si>
-  <si>
-    <t>2026-09-28T06:11:14.621Z</t>
+    <t>2026-09-28T08:41:15.257Z</t>
   </si>
   <si>
     <t>Climbing New Zealand</t>
@@ -178,13 +193,28 @@
     <t>https://wknd.site/us/en/adventures/climbing-new-zealand.html</t>
   </si>
   <si>
+    <t>us/en/adventures/cycling-southern-utah.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah</t>
+  </si>
+  <si>
+    <t>2026-09-28T08:41:46.894Z</t>
+  </si>
+  <si>
+    <t>Cycling Southern Utah</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/cycling-southern-utah.html</t>
+  </si>
+  <si>
     <t>us/en/adventures/downhill-skiing-wyoming.report.json</t>
   </si>
   <si>
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-09-28T06:11:19.916Z</t>
+    <t>2026-09-28T08:41:20.412Z</t>
   </si>
   <si>
     <t>Downhill Skiing Wyoming</t>
@@ -199,7 +229,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-09-28T06:11:26.660Z</t>
+    <t>2026-09-28T08:41:25.316Z</t>
   </si>
   <si>
     <t>Tahoe Skiing</t>
@@ -214,7 +244,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-09-28T06:11:32.880Z</t>
+    <t>2026-09-28T08:41:30.818Z</t>
   </si>
   <si>
     <t>West Coast Cycling</t>
@@ -232,7 +262,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-09-28T06:11:37.918Z</t>
+    <t>2026-09-28T08:41:36.824Z</t>
   </si>
   <si>
     <t>Whistler Mountain Biking</t>
@@ -247,7 +277,7 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-09-28T06:11:42.534Z</t>
+    <t>2026-09-28T08:41:41.885Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>
@@ -271,7 +301,7 @@
     <t>article</t>
   </si>
   <si>
-    <t>2026-09-28T05:59:42.238Z</t>
+    <t>2026-09-28T08:40:49.424Z</t>
   </si>
   <si>
     <t>Arctic Surfing</t>
@@ -289,7 +319,7 @@
     <t>us/en/magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>2026-09-28T05:59:48.423Z</t>
+    <t>2026-09-28T08:40:56.213Z</t>
   </si>
   <si>
     <t>Ultimate Guide to LA Skateparks</t>
@@ -304,7 +334,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-09-28T05:59:52.683Z</t>
+    <t>2026-09-28T08:41:01.781Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -322,7 +352,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-09-28T05:59:56.697Z</t>
+    <t>2026-09-28T08:41:06.680Z</t>
   </si>
   <si>
     <t>Ski Touring</t>
@@ -340,7 +370,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-09-28T05:59:37.701Z</t>
+    <t>2026-09-28T08:40:44.775Z</t>
   </si>
   <si>
     <t>Western Australia</t>
@@ -735,7 +765,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -925,39 +955,39 @@
         <v>47</v>
       </c>
       <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
         <v>48</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>49</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s">
         <v>50</v>
       </c>
-      <c r="E7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>51</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>52</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>53</v>
-      </c>
-      <c r="I7" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" t="s">
         <v>55</v>
       </c>
-      <c r="B8" t="s">
-        <v>19</v>
-      </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D8" t="s">
         <v>56</v>
@@ -966,7 +996,7 @@
         <v>13</v>
       </c>
       <c r="F8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G8" t="s">
         <v>57</v>
@@ -986,7 +1016,7 @@
         <v>19</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D9" t="s">
         <v>61</v>
@@ -995,7 +1025,7 @@
         <v>13</v>
       </c>
       <c r="F9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G9" t="s">
         <v>62</v>
@@ -1015,7 +1045,7 @@
         <v>19</v>
       </c>
       <c r="C10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D10" t="s">
         <v>66</v>
@@ -1024,7 +1054,7 @@
         <v>13</v>
       </c>
       <c r="F10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G10" t="s">
         <v>67</v>
@@ -1041,202 +1071,260 @@
         <v>70</v>
       </c>
       <c r="B11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" t="s">
         <v>71</v>
       </c>
-      <c r="C11" t="s">
-        <v>49</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" t="s">
+        <v>50</v>
+      </c>
+      <c r="G11" t="s">
         <v>72</v>
       </c>
-      <c r="E11" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" t="s">
-        <v>51</v>
-      </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>73</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>74</v>
-      </c>
-      <c r="I11" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
         <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D12" t="s">
+        <v>76</v>
+      </c>
+      <c r="E12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G12" t="s">
         <v>77</v>
       </c>
-      <c r="E12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" t="s">
-        <v>51</v>
-      </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>78</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>79</v>
-      </c>
-      <c r="I12" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>80</v>
+      </c>
+      <c r="B13" t="s">
         <v>81</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
+        <v>48</v>
+      </c>
+      <c r="D13" t="s">
         <v>82</v>
       </c>
-      <c r="C13" t="s">
+      <c r="E13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" t="s">
+        <v>50</v>
+      </c>
+      <c r="G13" t="s">
         <v>83</v>
       </c>
-      <c r="D13" t="s">
+      <c r="H13" t="s">
         <v>84</v>
       </c>
-      <c r="E13" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="I13" t="s">
         <v>85</v>
-      </c>
-      <c r="G13" t="s">
-        <v>86</v>
-      </c>
-      <c r="H13" t="s">
-        <v>87</v>
-      </c>
-      <c r="I13" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>86</v>
+      </c>
+      <c r="B14" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" t="s">
+        <v>87</v>
+      </c>
+      <c r="E14" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" t="s">
+        <v>50</v>
+      </c>
+      <c r="G14" t="s">
+        <v>88</v>
+      </c>
+      <c r="H14" t="s">
         <v>89</v>
       </c>
-      <c r="B14" t="s">
+      <c r="I14" t="s">
         <v>90</v>
-      </c>
-      <c r="C14" t="s">
-        <v>83</v>
-      </c>
-      <c r="D14" t="s">
-        <v>91</v>
-      </c>
-      <c r="E14" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" t="s">
-        <v>85</v>
-      </c>
-      <c r="G14" t="s">
-        <v>92</v>
-      </c>
-      <c r="H14" t="s">
-        <v>93</v>
-      </c>
-      <c r="I14" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" t="s">
+        <v>92</v>
+      </c>
+      <c r="C15" t="s">
+        <v>93</v>
+      </c>
+      <c r="D15" t="s">
+        <v>94</v>
+      </c>
+      <c r="E15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s">
         <v>95</v>
       </c>
-      <c r="B15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" t="s">
-        <v>83</v>
-      </c>
-      <c r="D15" t="s">
+      <c r="G15" t="s">
         <v>96</v>
       </c>
-      <c r="E15" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" t="s">
-        <v>85</v>
-      </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>97</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>98</v>
-      </c>
-      <c r="I15" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>99</v>
+      </c>
+      <c r="B16" t="s">
         <v>100</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
+        <v>93</v>
+      </c>
+      <c r="D16" t="s">
         <v>101</v>
       </c>
-      <c r="C16" t="s">
-        <v>83</v>
-      </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" t="s">
+        <v>95</v>
+      </c>
+      <c r="G16" t="s">
         <v>102</v>
       </c>
-      <c r="E16" t="s">
-        <v>13</v>
-      </c>
-      <c r="F16" t="s">
-        <v>85</v>
-      </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>103</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>104</v>
-      </c>
-      <c r="I16" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>105</v>
+      </c>
+      <c r="B17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" t="s">
+        <v>93</v>
+      </c>
+      <c r="D17" t="s">
         <v>106</v>
       </c>
-      <c r="B17" t="s">
+      <c r="E17" t="s">
+        <v>13</v>
+      </c>
+      <c r="F17" t="s">
+        <v>95</v>
+      </c>
+      <c r="G17" t="s">
         <v>107</v>
       </c>
-      <c r="C17" t="s">
-        <v>83</v>
-      </c>
-      <c r="D17" t="s">
+      <c r="H17" t="s">
         <v>108</v>
       </c>
-      <c r="E17" t="s">
-        <v>13</v>
-      </c>
-      <c r="F17" t="s">
-        <v>85</v>
-      </c>
-      <c r="G17" t="s">
+      <c r="I17" t="s">
         <v>109</v>
       </c>
-      <c r="H17" t="s">
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>110</v>
       </c>
-      <c r="I17" t="s">
+      <c r="B18" t="s">
         <v>111</v>
+      </c>
+      <c r="C18" t="s">
+        <v>93</v>
+      </c>
+      <c r="D18" t="s">
+        <v>112</v>
+      </c>
+      <c r="E18" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" t="s">
+        <v>95</v>
+      </c>
+      <c r="G18" t="s">
+        <v>113</v>
+      </c>
+      <c r="H18" t="s">
+        <v>114</v>
+      </c>
+      <c r="I18" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>116</v>
+      </c>
+      <c r="B19" t="s">
+        <v>117</v>
+      </c>
+      <c r="C19" t="s">
+        <v>93</v>
+      </c>
+      <c r="D19" t="s">
+        <v>118</v>
+      </c>
+      <c r="E19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" t="s">
+        <v>95</v>
+      </c>
+      <c r="G19" t="s">
+        <v>119</v>
+      </c>
+      <c r="H19" t="s">
+        <v>120</v>
+      </c>
+      <c r="I19" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>